<commit_message>
Changes made due to UI changes
</commit_message>
<xml_diff>
--- a/fedan_rates.xlsx
+++ b/fedan_rates.xlsx
@@ -379,7 +379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:N16"/>
+  <dimension ref="A1:N17"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.453125" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="6" customWidth="1" style="6" min="1" max="1"/>
@@ -647,18 +647,34 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="6" t="n">
         <v>7</v>
       </c>
       <c r="B16" s="11" t="n">
         <v>46275</v>
       </c>
-      <c r="I16" t="n">
+      <c r="I16" s="6" t="n">
         <v>152.14</v>
       </c>
-      <c r="J16" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>2026-09-10 14:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>8</v>
+      </c>
+      <c r="B17" s="11" t="n">
+        <v>46293</v>
+      </c>
+      <c r="C17" t="n">
+        <v>153.19</v>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>2026-09-28 11:10</t>
         </is>
       </c>
     </row>

</xml_diff>